<commit_message>
edited excel report sytling
</commit_message>
<xml_diff>
--- a/backend/State of the Market Report - Nov 2023.xlsx
+++ b/backend/State of the Market Report - Nov 2023.xlsx
@@ -149,13 +149,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -499,7 +502,10 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="6" width="9" style="1" customWidth="1"/>
+    <col min="1" max="1" width="35" style="1" customWidth="1"/>
+    <col min="2" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="5" width="9" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -512,24 +518,24 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="2">
@@ -538,18 +544,18 @@
       <c r="E2" s="2">
         <v>4.8</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="3">
         <v>-0.016666666666666684</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="2">
@@ -558,18 +564,18 @@
       <c r="E3" s="2">
         <v>5.33</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="2">
@@ -578,18 +584,18 @@
       <c r="E4" s="2">
         <v>310.16</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="3">
         <v>0.004320350786690659</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="2">
@@ -598,18 +604,18 @@
       <c r="E5" s="2">
         <v>3.8</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="3">
         <v>0.026315789473684237</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="2">
@@ -618,18 +624,18 @@
       <c r="E6" s="2">
         <v>306.27</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="3">
         <v>0.003950762399190376</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="2">
@@ -638,18 +644,18 @@
       <c r="E7" s="2">
         <v>18714.7</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="3">
         <v>0.007411286315035813</v>
       </c>
     </row>
-    <row r="8" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="2">
@@ -658,18 +664,18 @@
       <c r="E8" s="2">
         <v>9497</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="3">
         <v>0.005896598925976624</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="2">
@@ -678,18 +684,18 @@
       <c r="E9" s="2">
         <v>3.7</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="2">
@@ -698,18 +704,18 @@
       <c r="E10" s="2">
         <v>3.6</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="3">
         <v>-0.0277777777777778</v>
       </c>
     </row>
-    <row r="11" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="2">
@@ -718,18 +724,18 @@
       <c r="E11" s="2">
         <v>4</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="3">
         <v>-0.15000000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="2">
@@ -738,7 +744,7 @@
       <c r="E12" s="2">
         <v>98</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="3">
         <v>0</v>
       </c>
     </row>
@@ -753,7 +759,8 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="9" style="1" customWidth="1"/>
+    <col min="1" max="1" width="30" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>